<commit_message>
HW updates over the past couple of weeks.
</commit_message>
<xml_diff>
--- a/HW10/DebiGonzalez_HW10_Interactions_PartII.xlsx
+++ b/HW10/DebiGonzalez_HW10_Interactions_PartII.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/debig/Documents/PhD Y1/Stats II/Quant II Projects/HW9/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/debig/Documents/PhD Y1/Stats II/Quant II Projects/HW10/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61826FD6-964B-B74C-A057-39DBA62459B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE1AD4E7-4B54-3C4C-AE15-BBB632004373}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1160" yWindow="500" windowWidth="27640" windowHeight="16040" xr2:uid="{C0996B5F-21C7-9B4B-99AB-F21C606EBDF2}"/>
   </bookViews>
@@ -47,9 +47,6 @@
     <t>Simple Slope Deltay/deltax</t>
   </si>
   <si>
-    <t>(Constant)</t>
-  </si>
-  <si>
     <t>b0</t>
   </si>
   <si>
@@ -71,15 +68,6 @@
     <t>$B$10+$B$11*C$1+$B$12*$A2+$B$13*C$1*$A2</t>
   </si>
   <si>
-    <t>hrs</t>
-  </si>
-  <si>
-    <t>advisorSupport</t>
-  </si>
-  <si>
-    <t>hrsXadvisorSupport</t>
-  </si>
-  <si>
     <t>Advisor Support Moderator</t>
   </si>
   <si>
@@ -90,6 +78,18 @@
   </si>
   <si>
     <t>High Advisor Support (+1 SD)</t>
+  </si>
+  <si>
+    <t>hrs_z</t>
+  </si>
+  <si>
+    <t>(Intercept)</t>
+  </si>
+  <si>
+    <t>advisorSupport_z</t>
+  </si>
+  <si>
+    <t>hrs_zXadvisorSupport_z</t>
   </si>
 </sst>
 </file>
@@ -295,19 +295,19 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>5.2664130399519999</c:v>
+                  <c:v>-1.0965100000000001</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>5.155263715856</c:v>
+                  <c:v>-1.7901400000000001</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>5.0441143917599991</c:v>
+                  <c:v>-2.4837699999999998</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>4.9329650676639991</c:v>
+                  <c:v>-3.1773999999999996</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>4.8218157435679991</c:v>
+                  <c:v>-3.8710299999999997</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -376,19 +376,19 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>3.2031294879999996</c:v>
+                  <c:v>-0.44494</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>3.144474464</c:v>
+                  <c:v>-0.81097999999999992</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>3.0858194399999999</c:v>
+                  <c:v>-1.17702</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>3.0271644159999997</c:v>
+                  <c:v>-1.5430599999999999</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>2.9685093919999996</c:v>
+                  <c:v>-1.9090999999999998</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -457,19 +457,19 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>1.1398459360479998</c:v>
+                  <c:v>0.20662999999999998</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1.1336852121440002</c:v>
+                  <c:v>0.16818000000000005</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1.1275244882400002</c:v>
+                  <c:v>0.1297299999999999</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>1.1213637643359999</c:v>
+                  <c:v>9.1280000000000028E-2</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>1.1152030404319997</c:v>
+                  <c:v>5.2830000000000155E-2</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -500,6 +500,66 @@
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="b"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Number of Hours Worked in</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="en-US" baseline="0"/>
+                  <a:t> Standard Deviation Units</a:t>
+                </a:r>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
@@ -1634,178 +1694,178 @@
     <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2">
         <f>D11-E11</f>
-        <v>-1.2527519999999999</v>
+        <v>-1</v>
       </c>
       <c r="B2" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="C2">
         <f>$B$10+$B$11*C$1+$B$12*$A2+$B$13*C$1*$A2</f>
-        <v>5.2664130399519999</v>
+        <v>-1.0965100000000001</v>
       </c>
       <c r="D2">
         <f t="shared" ref="D2:G2" si="0">$B$10+$B$11*D$1+$B$12*$A2+$B$13*D$1*$A2</f>
-        <v>5.155263715856</v>
+        <v>-1.7901400000000001</v>
       </c>
       <c r="E2">
         <f t="shared" si="0"/>
-        <v>5.0441143917599991</v>
+        <v>-2.4837699999999998</v>
       </c>
       <c r="F2">
         <f t="shared" si="0"/>
-        <v>4.9329650676639991</v>
+        <v>-3.1773999999999996</v>
       </c>
       <c r="G2">
         <f t="shared" si="0"/>
-        <v>4.8218157435679991</v>
+        <v>-3.8710299999999997</v>
       </c>
       <c r="H2">
         <f>$B$11+$B$13*$A2</f>
-        <v>-0.11114932409600001</v>
+        <v>-0.69362999999999997</v>
       </c>
       <c r="I2">
         <f>D2-C2</f>
-        <v>-0.11114932409599998</v>
+        <v>-0.69362999999999997</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3">
         <f>D11</f>
-        <v>0.312</v>
+        <v>0</v>
       </c>
       <c r="B3" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="C3">
         <f t="shared" ref="C3:G4" si="1">$B$10+$B$11*C$1+$B$12*$A3+$B$13*C$1*$A3</f>
-        <v>3.2031294879999996</v>
+        <v>-0.44494</v>
       </c>
       <c r="D3">
         <f t="shared" si="1"/>
-        <v>3.144474464</v>
+        <v>-0.81097999999999992</v>
       </c>
       <c r="E3">
         <f t="shared" si="1"/>
-        <v>3.0858194399999999</v>
+        <v>-1.17702</v>
       </c>
       <c r="F3">
         <f t="shared" si="1"/>
-        <v>3.0271644159999997</v>
+        <v>-1.5430599999999999</v>
       </c>
       <c r="G3">
         <f t="shared" si="1"/>
-        <v>2.9685093919999996</v>
+        <v>-1.9090999999999998</v>
       </c>
       <c r="H3">
         <f t="shared" ref="H3:H4" si="2">$B$11+$B$13*$A3</f>
-        <v>-5.8655024E-2</v>
+        <v>-0.36603999999999998</v>
       </c>
       <c r="I3">
         <f t="shared" ref="I3:I4" si="3">D3-C3</f>
-        <v>-5.8655023999999667E-2</v>
+        <v>-0.36603999999999992</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4">
         <f>D11+E11</f>
-        <v>1.876752</v>
+        <v>1</v>
       </c>
       <c r="B4" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="C4">
         <f t="shared" si="1"/>
-        <v>1.1398459360479998</v>
+        <v>0.20662999999999998</v>
       </c>
       <c r="D4">
         <f t="shared" si="1"/>
-        <v>1.1336852121440002</v>
+        <v>0.16818000000000005</v>
       </c>
       <c r="E4">
         <f t="shared" si="1"/>
-        <v>1.1275244882400002</v>
+        <v>0.1297299999999999</v>
       </c>
       <c r="F4">
         <f t="shared" si="1"/>
-        <v>1.1213637643359999</v>
+        <v>9.1280000000000028E-2</v>
       </c>
       <c r="G4">
         <f t="shared" si="1"/>
-        <v>1.1152030404319997</v>
+        <v>5.2830000000000155E-2</v>
       </c>
       <c r="H4">
         <f t="shared" si="2"/>
-        <v>-6.1607239040000067E-3</v>
+        <v>-3.8449999999999984E-2</v>
       </c>
       <c r="I4">
-        <f t="shared" si="3"/>
-        <v>-6.1607239039995765E-3</v>
+        <f>D4-C4</f>
+        <v>-3.8449999999999929E-2</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.2">
       <c r="D9" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B10" s="2">
+        <v>-7.8899999999999998E-2</v>
+      </c>
+      <c r="C10" t="s">
         <v>3</v>
       </c>
-      <c r="B10" s="2">
-        <v>3.6836549999999999</v>
-      </c>
-      <c r="C10" t="s">
+      <c r="D10" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D10" s="1" t="s">
+      <c r="E10" s="1" t="s">
         <v>5</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B11" s="2">
-        <v>-6.9122000000000003E-2</v>
+        <v>-0.36603999999999998</v>
       </c>
       <c r="C11" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D11" s="2">
-        <v>0.312</v>
+        <v>0</v>
       </c>
       <c r="E11" s="2">
-        <v>1.5647519999999999</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="B12" s="2">
-        <v>-1.352149</v>
+        <v>0.32397999999999999</v>
       </c>
       <c r="C12" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B13" s="2">
-        <v>3.3548000000000001E-2</v>
+        <v>0.32758999999999999</v>
       </c>
       <c r="C13" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>